<commit_message>
data: 更新淨值表至 2026-07-15（via Portal）
</commit_message>
<xml_diff>
--- a/assets/data/Yi_Capital_US.xlsx
+++ b/assets/data/Yi_Capital_US.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2149,7 +2149,7 @@
       </c>
       <c r="E55" s="2" t="n"/>
       <c r="F55" s="4" t="n">
-        <v>1388</v>
+        <v>2809.86</v>
       </c>
       <c r="G55" s="2" t="n"/>
       <c r="H55" s="2" t="n"/>
@@ -2234,6 +2234,39 @@
         <v>138.8</v>
       </c>
       <c r="I57" s="7" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Oracle Corporation</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="F58" s="9" t="n">
+        <v>1421.86</v>
+      </c>
+      <c r="G58" s="10" t="n">
+        <v>129.26</v>
+      </c>
+      <c r="H58" s="10" t="n">
+        <v>129.26</v>
+      </c>
+      <c r="I58" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -2260,7 +2293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F103"/>
+  <dimension ref="A1:F110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4706,12 +4739,12 @@
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B102" s="7" t="inlineStr">
         <is>
-          <t>ETF Stock Buy Record</t>
+          <t>ETF Stock Dividend Record</t>
         </is>
       </c>
       <c r="C102" s="7" t="n">
@@ -4721,10 +4754,10 @@
         <v>-16538.54</v>
       </c>
       <c r="E102" s="9" t="n">
-        <v>-1388</v>
+        <v>61.23</v>
       </c>
       <c r="F102" s="9" t="n">
-        <v>-17926.54</v>
+        <v>-16477.31</v>
       </c>
     </row>
     <row r="103">
@@ -4735,20 +4768,188 @@
       </c>
       <c r="B103" s="7" t="inlineStr">
         <is>
-          <t>ETF Stock Sell Record</t>
+          <t>ETF Stock Buy Record</t>
         </is>
       </c>
       <c r="C103" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D103" s="9" t="n">
-        <v>-17926.54</v>
+        <v>-16477.31</v>
       </c>
       <c r="E103" s="9" t="n">
+        <v>-1388</v>
+      </c>
+      <c r="F103" s="9" t="n">
+        <v>-17865.31</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B104" s="7" t="inlineStr">
+        <is>
+          <t>ETF Stock Sell Record</t>
+        </is>
+      </c>
+      <c r="C104" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D104" s="9" t="n">
+        <v>-17865.31</v>
+      </c>
+      <c r="E104" s="9" t="n">
         <v>406.8</v>
       </c>
-      <c r="F103" s="9" t="n">
-        <v>-17519.74</v>
+      <c r="F104" s="9" t="n">
+        <v>-17458.51</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B105" s="7" t="inlineStr">
+        <is>
+          <t>ETF Stock Sell Record</t>
+        </is>
+      </c>
+      <c r="C105" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D105" s="9" t="n">
+        <v>-17458.51</v>
+      </c>
+      <c r="E105" s="9" t="n">
+        <v>363.96</v>
+      </c>
+      <c r="F105" s="9" t="n">
+        <v>-17094.55</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr">
+        <is>
+          <t>ETF Stock Dividend Record</t>
+        </is>
+      </c>
+      <c r="C106" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D106" s="9" t="n">
+        <v>-17094.55</v>
+      </c>
+      <c r="E106" s="9" t="n">
+        <v>44.53</v>
+      </c>
+      <c r="F106" s="9" t="n">
+        <v>-17050.02</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B107" s="7" t="inlineStr">
+        <is>
+          <t>ETF Stock Dividend Record</t>
+        </is>
+      </c>
+      <c r="C107" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D107" s="9" t="n">
+        <v>-17050.02</v>
+      </c>
+      <c r="E107" s="9" t="n">
+        <v>31.05</v>
+      </c>
+      <c r="F107" s="9" t="n">
+        <v>-17018.97</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B108" s="7" t="inlineStr">
+        <is>
+          <t>ETF Stock Dividend Record</t>
+        </is>
+      </c>
+      <c r="C108" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D108" s="9" t="n">
+        <v>-17018.97</v>
+      </c>
+      <c r="E108" s="9" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="F108" s="9" t="n">
+        <v>-17017.22</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B109" s="7" t="inlineStr">
+        <is>
+          <t>ETF Stock Buy Record</t>
+        </is>
+      </c>
+      <c r="C109" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D109" s="9" t="n">
+        <v>-17017.22</v>
+      </c>
+      <c r="E109" s="9" t="n">
+        <v>-1421.86</v>
+      </c>
+      <c r="F109" s="9" t="n">
+        <v>-18439.08</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B110" s="7" t="inlineStr">
+        <is>
+          <t>ETF Stock Sell Record</t>
+        </is>
+      </c>
+      <c r="C110" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D110" s="9" t="n">
+        <v>-18439.08</v>
+      </c>
+      <c r="E110" s="9" t="n">
+        <v>5630</v>
+      </c>
+      <c r="F110" s="9" t="n">
+        <v>-12809.08</v>
       </c>
     </row>
   </sheetData>
@@ -4762,7 +4963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J132"/>
+  <dimension ref="A1:J133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5074,7 +5275,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>153121.43</v>
+        <v>153121.44</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>0</v>
@@ -5083,7 +5284,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>153121.43</v>
+        <v>153121.44</v>
       </c>
       <c r="F9" s="8" t="n">
         <v>1513476.32</v>
@@ -5098,7 +5299,7 @@
         <v>13619.69</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>139501.74</v>
+        <v>139501.75</v>
       </c>
     </row>
     <row r="10">
@@ -5108,7 +5309,7 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>153368.67</v>
+        <v>153368.68</v>
       </c>
       <c r="C10" s="9" t="n">
         <v>0</v>
@@ -5117,7 +5318,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>153368.67</v>
+        <v>153368.68</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>1513476.32</v>
@@ -5132,7 +5333,7 @@
         <v>13619.69</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>139748.98</v>
+        <v>139748.99</v>
       </c>
     </row>
     <row r="11">
@@ -5414,7 +5615,7 @@
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>155929.19</v>
+        <v>155929.2</v>
       </c>
       <c r="C19" s="9" t="n">
         <v>0</v>
@@ -5423,7 +5624,7 @@
         <v>0</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>155929.19</v>
+        <v>155929.2</v>
       </c>
       <c r="F19" s="8" t="n">
         <v>1513476.32</v>
@@ -5438,7 +5639,7 @@
         <v>27249.8</v>
       </c>
       <c r="J19" s="9" t="n">
-        <v>128679.39</v>
+        <v>128679.4</v>
       </c>
     </row>
     <row r="20">
@@ -5448,7 +5649,7 @@
         </is>
       </c>
       <c r="B20" s="9" t="n">
-        <v>205195.01</v>
+        <v>205195.02</v>
       </c>
       <c r="C20" s="9" t="n">
         <v>0</v>
@@ -5457,7 +5658,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>205195.01</v>
+        <v>205195.02</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>2005476.32</v>
@@ -5472,7 +5673,7 @@
         <v>39507.2</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>165687.81</v>
+        <v>165687.82</v>
       </c>
     </row>
     <row r="21">
@@ -5550,7 +5751,7 @@
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>208407.89</v>
+        <v>208407.9</v>
       </c>
       <c r="C23" s="9" t="n">
         <v>0</v>
@@ -5559,7 +5760,7 @@
         <v>0</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>208407.89</v>
+        <v>208407.9</v>
       </c>
       <c r="F23" s="8" t="n">
         <v>2054841.55</v>
@@ -5574,7 +5775,7 @@
         <v>13000.1</v>
       </c>
       <c r="J23" s="9" t="n">
-        <v>195407.79</v>
+        <v>195407.8</v>
       </c>
     </row>
     <row r="24">
@@ -5584,7 +5785,7 @@
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>206929.19</v>
+        <v>206929.2</v>
       </c>
       <c r="C24" s="9" t="n">
         <v>0</v>
@@ -5593,7 +5794,7 @@
         <v>0</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>206929.19</v>
+        <v>206929.2</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>2054841.55</v>
@@ -5608,7 +5809,7 @@
         <v>13000.1</v>
       </c>
       <c r="J24" s="9" t="n">
-        <v>193929.09</v>
+        <v>193929.1</v>
       </c>
     </row>
     <row r="25">
@@ -5686,7 +5887,7 @@
         </is>
       </c>
       <c r="B27" s="9" t="n">
-        <v>215332.61</v>
+        <v>215332.6</v>
       </c>
       <c r="C27" s="9" t="n">
         <v>0</v>
@@ -5695,7 +5896,7 @@
         <v>0</v>
       </c>
       <c r="E27" s="9" t="n">
-        <v>215332.61</v>
+        <v>215332.6</v>
       </c>
       <c r="F27" s="8" t="n">
         <v>2107072.57</v>
@@ -5710,7 +5911,7 @@
         <v>0</v>
       </c>
       <c r="J27" s="9" t="n">
-        <v>215332.61</v>
+        <v>215332.6</v>
       </c>
     </row>
     <row r="28">
@@ -5720,7 +5921,7 @@
         </is>
       </c>
       <c r="B28" s="9" t="n">
-        <v>214482.65</v>
+        <v>214482.66</v>
       </c>
       <c r="C28" s="9" t="n">
         <v>0</v>
@@ -5729,7 +5930,7 @@
         <v>0</v>
       </c>
       <c r="E28" s="9" t="n">
-        <v>214482.65</v>
+        <v>214482.66</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>2107072.57</v>
@@ -5744,7 +5945,7 @@
         <v>0</v>
       </c>
       <c r="J28" s="9" t="n">
-        <v>214482.65</v>
+        <v>214482.66</v>
       </c>
     </row>
     <row r="29">
@@ -5822,7 +6023,7 @@
         </is>
       </c>
       <c r="B31" s="9" t="n">
-        <v>212741.95</v>
+        <v>212741.94</v>
       </c>
       <c r="C31" s="9" t="n">
         <v>0</v>
@@ -5831,7 +6032,7 @@
         <v>0</v>
       </c>
       <c r="E31" s="9" t="n">
-        <v>212741.95</v>
+        <v>212741.94</v>
       </c>
       <c r="F31" s="8" t="n">
         <v>2107072.57</v>
@@ -5846,7 +6047,7 @@
         <v>0</v>
       </c>
       <c r="J31" s="9" t="n">
-        <v>212741.95</v>
+        <v>212741.94</v>
       </c>
     </row>
     <row r="32">
@@ -6876,7 +7077,7 @@
         </is>
       </c>
       <c r="B62" s="9" t="n">
-        <v>212156.27</v>
+        <v>212156.26</v>
       </c>
       <c r="C62" s="9" t="n">
         <v>0</v>
@@ -6885,7 +7086,7 @@
         <v>0</v>
       </c>
       <c r="E62" s="9" t="n">
-        <v>212156.27</v>
+        <v>212156.26</v>
       </c>
       <c r="F62" s="8" t="n">
         <v>2107072.57</v>
@@ -6900,7 +7101,7 @@
         <v>-5732.01</v>
       </c>
       <c r="J62" s="9" t="n">
-        <v>217888.28</v>
+        <v>217888.27</v>
       </c>
     </row>
     <row r="63">
@@ -7046,7 +7247,7 @@
         </is>
       </c>
       <c r="B67" s="9" t="n">
-        <v>213605</v>
+        <v>213604.99</v>
       </c>
       <c r="C67" s="9" t="n">
         <v>0</v>
@@ -7055,7 +7256,7 @@
         <v>0</v>
       </c>
       <c r="E67" s="9" t="n">
-        <v>213605</v>
+        <v>213604.99</v>
       </c>
       <c r="F67" s="8" t="n">
         <v>2107072.57</v>
@@ -7070,7 +7271,7 @@
         <v>-5521.95</v>
       </c>
       <c r="J67" s="9" t="n">
-        <v>219126.95</v>
+        <v>219126.94</v>
       </c>
     </row>
     <row r="68">
@@ -9052,7 +9253,7 @@
         </is>
       </c>
       <c r="B126" s="9" t="n">
-        <v>221887.09</v>
+        <v>221948.32</v>
       </c>
       <c r="C126" s="9" t="n">
         <v>0</v>
@@ -9061,19 +9262,19 @@
         <v>0</v>
       </c>
       <c r="E126" s="9" t="n">
-        <v>221887.09</v>
+        <v>221948.32</v>
       </c>
       <c r="F126" s="8" t="n">
         <v>2107072.57</v>
       </c>
       <c r="G126" s="16" t="n">
-        <v>0.105306</v>
+        <v>0.105335</v>
       </c>
       <c r="H126" s="9" t="n">
         <v>-0</v>
       </c>
       <c r="I126" s="9" t="n">
-        <v>-16538.54</v>
+        <v>-16477.31</v>
       </c>
       <c r="J126" s="9" t="n">
         <v>238425.63</v>
@@ -9086,7 +9287,7 @@
         </is>
       </c>
       <c r="B127" s="9" t="n">
-        <v>223453.64</v>
+        <v>223514.87</v>
       </c>
       <c r="C127" s="9" t="n">
         <v>0</v>
@@ -9095,19 +9296,19 @@
         <v>0</v>
       </c>
       <c r="E127" s="9" t="n">
-        <v>223453.64</v>
+        <v>223514.87</v>
       </c>
       <c r="F127" s="8" t="n">
         <v>2107072.57</v>
       </c>
       <c r="G127" s="16" t="n">
-        <v>0.106049</v>
+        <v>0.106078</v>
       </c>
       <c r="H127" s="9" t="n">
         <v>-0</v>
       </c>
       <c r="I127" s="9" t="n">
-        <v>-17519.74</v>
+        <v>-17458.51</v>
       </c>
       <c r="J127" s="9" t="n">
         <v>240973.38</v>
@@ -9120,7 +9321,7 @@
         </is>
       </c>
       <c r="B128" s="9" t="n">
-        <v>221746.61</v>
+        <v>221829.33</v>
       </c>
       <c r="C128" s="9" t="n">
         <v>0</v>
@@ -9129,22 +9330,22 @@
         <v>0</v>
       </c>
       <c r="E128" s="9" t="n">
-        <v>221746.61</v>
+        <v>221829.33</v>
       </c>
       <c r="F128" s="8" t="n">
         <v>2107072.57</v>
       </c>
       <c r="G128" s="16" t="n">
-        <v>0.105239</v>
+        <v>0.105278</v>
       </c>
       <c r="H128" s="9" t="n">
         <v>-0</v>
       </c>
       <c r="I128" s="9" t="n">
-        <v>-17519.74</v>
+        <v>-17050.02</v>
       </c>
       <c r="J128" s="9" t="n">
-        <v>239266.35</v>
+        <v>238879.35</v>
       </c>
     </row>
     <row r="129">
@@ -9154,7 +9355,7 @@
         </is>
       </c>
       <c r="B129" s="9" t="n">
-        <v>222272.13</v>
+        <v>222341.17</v>
       </c>
       <c r="C129" s="9" t="n">
         <v>0</v>
@@ -9163,22 +9364,22 @@
         <v>0</v>
       </c>
       <c r="E129" s="9" t="n">
-        <v>222272.13</v>
+        <v>222341.17</v>
       </c>
       <c r="F129" s="8" t="n">
         <v>2107072.57</v>
       </c>
       <c r="G129" s="16" t="n">
-        <v>0.105489</v>
+        <v>0.105521</v>
       </c>
       <c r="H129" s="9" t="n">
         <v>-0</v>
       </c>
       <c r="I129" s="9" t="n">
-        <v>-17519.74</v>
+        <v>-17050.02</v>
       </c>
       <c r="J129" s="9" t="n">
-        <v>239791.87</v>
+        <v>239391.19</v>
       </c>
     </row>
     <row r="130">
@@ -9188,7 +9389,7 @@
         </is>
       </c>
       <c r="B130" s="9" t="n">
-        <v>223492</v>
+        <v>223618.37</v>
       </c>
       <c r="C130" s="9" t="n">
         <v>0</v>
@@ -9197,22 +9398,22 @@
         <v>0</v>
       </c>
       <c r="E130" s="9" t="n">
-        <v>223492</v>
+        <v>223618.37</v>
       </c>
       <c r="F130" s="8" t="n">
         <v>2107072.57</v>
       </c>
       <c r="G130" s="16" t="n">
-        <v>0.106068</v>
+        <v>0.106128</v>
       </c>
       <c r="H130" s="9" t="n">
         <v>-0</v>
       </c>
       <c r="I130" s="9" t="n">
-        <v>-17519.74</v>
+        <v>-17018.97</v>
       </c>
       <c r="J130" s="9" t="n">
-        <v>241011.74</v>
+        <v>240637.34</v>
       </c>
     </row>
     <row r="131">
@@ -9222,7 +9423,7 @@
         </is>
       </c>
       <c r="B131" s="9" t="n">
-        <v>225633.76</v>
+        <v>225771.6</v>
       </c>
       <c r="C131" s="9" t="n">
         <v>0</v>
@@ -9231,22 +9432,22 @@
         <v>0</v>
       </c>
       <c r="E131" s="9" t="n">
-        <v>225633.76</v>
+        <v>225771.6</v>
       </c>
       <c r="F131" s="8" t="n">
         <v>2107072.57</v>
       </c>
       <c r="G131" s="16" t="n">
-        <v>0.107084</v>
+        <v>0.107149</v>
       </c>
       <c r="H131" s="9" t="n">
         <v>-0</v>
       </c>
       <c r="I131" s="9" t="n">
-        <v>-17519.74</v>
+        <v>-17017.22</v>
       </c>
       <c r="J131" s="9" t="n">
-        <v>243153.5</v>
+        <v>242788.82</v>
       </c>
     </row>
     <row r="132">
@@ -9256,7 +9457,7 @@
         </is>
       </c>
       <c r="B132" s="9" t="n">
-        <v>225633.76</v>
+        <v>223868.53</v>
       </c>
       <c r="C132" s="9" t="n">
         <v>0</v>
@@ -9265,22 +9466,56 @@
         <v>0</v>
       </c>
       <c r="E132" s="9" t="n">
-        <v>225633.76</v>
+        <v>223868.53</v>
       </c>
       <c r="F132" s="8" t="n">
         <v>2107072.57</v>
       </c>
       <c r="G132" s="16" t="n">
-        <v>0.107084</v>
+        <v>0.106246</v>
       </c>
       <c r="H132" s="9" t="n">
         <v>-0</v>
       </c>
       <c r="I132" s="9" t="n">
-        <v>-17519.74</v>
+        <v>-18439.08</v>
       </c>
       <c r="J132" s="9" t="n">
-        <v>243153.5</v>
+        <v>242307.61</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B133" s="9" t="n">
+        <v>228717</v>
+      </c>
+      <c r="C133" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D133" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E133" s="9" t="n">
+        <v>228717</v>
+      </c>
+      <c r="F133" s="8" t="n">
+        <v>2107072.57</v>
+      </c>
+      <c r="G133" s="16" t="n">
+        <v>0.108547</v>
+      </c>
+      <c r="H133" s="9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I133" s="9" t="n">
+        <v>-12809.08</v>
+      </c>
+      <c r="J133" s="9" t="n">
+        <v>241526.08</v>
       </c>
     </row>
   </sheetData>
@@ -9294,7 +9529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10424,7 +10659,7 @@
       </c>
       <c r="E40" s="2" t="n"/>
       <c r="F40" s="4" t="n">
-        <v>406.8</v>
+        <v>6400.76</v>
       </c>
       <c r="G40" s="2" t="n"/>
       <c r="H40" s="2" t="n"/>
@@ -10509,6 +10744,72 @@
         <v>20.34</v>
       </c>
       <c r="I42" s="7" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>MBGL</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>Mobility Global Inc.</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="F43" s="9" t="n">
+        <v>363.96</v>
+      </c>
+      <c r="G43" s="10" t="n">
+        <v>20.22</v>
+      </c>
+      <c r="H43" s="10" t="n">
+        <v>20.22</v>
+      </c>
+      <c r="I43" s="7" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>PayPal Holdings, Inc.</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="F44" s="9" t="n">
+        <v>5630</v>
+      </c>
+      <c r="G44" s="10" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="H44" s="10" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="I44" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -10537,7 +10838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11882,11 +12183,195 @@
       </c>
       <c r="H49" s="7" t="n"/>
     </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>2026/07/01-2026/07/31</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n"/>
+      <c r="C51" s="2" t="n"/>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Total Dividend Amount:</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="4" t="n">
+        <v>138.56</v>
+      </c>
+      <c r="G51" s="2" t="n"/>
+      <c r="H51" s="2" t="n"/>
+    </row>
+    <row r="52" ht="28" customHeight="1">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Trade No.</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Execution Date</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Stock/ETF Name</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>Amount (USD)</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>Div Per Share (USD)</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>PBR-A</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Petrobras (Preferred ADR)</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="F53" s="9" t="n">
+        <v>61.23</v>
+      </c>
+      <c r="G53" s="10" t="n">
+        <v>0.10205</v>
+      </c>
+      <c r="H53" s="7" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>TLT</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>iShares 20+ Year Treasury Bond ETF</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="F54" s="9" t="n">
+        <v>44.53</v>
+      </c>
+      <c r="G54" s="10" t="n">
+        <v>0.22265</v>
+      </c>
+      <c r="H54" s="7" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>SGOV</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>iShares 0-3 Month Treasury Bond ETF</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="F55" s="9" t="n">
+        <v>31.05</v>
+      </c>
+      <c r="G55" s="10" t="n">
+        <v>0.207</v>
+      </c>
+      <c r="H55" s="7" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>PGR</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>The Progressive Corporation</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="F56" s="9" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="G56" s="10" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="H56" s="7" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="14">
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="D39:E39"/>
     <mergeCell ref="D1:E1"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="D51:E51"/>
     <mergeCell ref="D23:E23"/>
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="D32:E32"/>
@@ -12057,7 +12542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -12085,7 +12570,7 @@
       </c>
       <c r="B1" s="12" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="C1" s="2" t="n"/>
@@ -12103,7 +12588,7 @@
       </c>
       <c r="L1" s="2" t="n"/>
       <c r="M1" s="4" t="n">
-        <v>240276.88</v>
+        <v>241526.45</v>
       </c>
       <c r="N1" s="2" t="n"/>
       <c r="O1" s="2" t="n"/>
@@ -12203,13 +12688,13 @@
         <v>20</v>
       </c>
       <c r="E3" s="10" t="n">
-        <v>428.1900024414062</v>
+        <v>423.1400146484375</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>8563.800048828125</v>
+        <v>8462.80029296875</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>0.03564138202803051</v>
+        <v>0.03503881394080345</v>
       </c>
       <c r="H3" s="9" t="n">
         <v>6893.1</v>
@@ -12224,13 +12709,13 @@
         <v>6893.1</v>
       </c>
       <c r="L3" s="9" t="n">
-        <v>1734.120048828125</v>
+        <v>1633.12029296875</v>
       </c>
       <c r="M3" s="15" t="n">
-        <v>0.2423728146738223</v>
+        <v>0.2277205165990265</v>
       </c>
       <c r="N3" s="15" t="n">
-        <v>0.2515733195265011</v>
+        <v>0.2369210214517053</v>
       </c>
       <c r="O3" s="7" t="n"/>
     </row>
@@ -12252,13 +12737,13 @@
         <v>150</v>
       </c>
       <c r="E4" s="10" t="n">
-        <v>74.33000183105469</v>
+        <v>73.59020233154297</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>11149.5002746582</v>
+        <v>11038.53034973145</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>0.04640271800426989</v>
+        <v>0.04570319488993528</v>
       </c>
       <c r="H4" s="9" t="n">
         <v>12219</v>
@@ -12273,13 +12758,13 @@
         <v>12219</v>
       </c>
       <c r="L4" s="9" t="n">
-        <v>-1069.499725341795</v>
+        <v>-1180.469650268553</v>
       </c>
       <c r="M4" s="15" t="n">
-        <v>-0.0875275984402812</v>
+        <v>-0.09660935021430181</v>
       </c>
       <c r="N4" s="15" t="n">
-        <v>-0.08752759844028114</v>
+        <v>-0.09660935021430175</v>
       </c>
       <c r="O4" s="7" t="n"/>
     </row>
@@ -12301,13 +12786,13 @@
         <v>20</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>377.489990234375</v>
+        <v>371.4349975585938</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>7549.7998046875</v>
+        <v>7428.699951171875</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>0.03142124962514032</v>
+        <v>0.03075729385076347</v>
       </c>
       <c r="H5" s="9" t="n">
         <v>22085.17</v>
@@ -12322,13 +12807,13 @@
         <v>9410.169999999998</v>
       </c>
       <c r="L5" s="9" t="n">
-        <v>-1860.370195312498</v>
+        <v>-1981.470048828123</v>
       </c>
       <c r="M5" s="15" t="n">
-        <v>-0.1976978306781385</v>
+        <v>-0.2105668706121275</v>
       </c>
       <c r="N5" s="15" t="n">
-        <v>-0.08423617274906638</v>
+        <v>-0.08971948365478388</v>
       </c>
       <c r="O5" s="7" t="n"/>
     </row>
@@ -12350,13 +12835,13 @@
         <v>600</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>14.98999977111816</v>
+        <v>15.85999965667725</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>8993.999862670898</v>
+        <v>9515.999794006348</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>0.03743181569370865</v>
+        <v>0.03939941091602262</v>
       </c>
       <c r="H6" s="9" t="n">
         <v>11165</v>
@@ -12365,19 +12850,19 @@
         <v>6936</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>229.77</v>
+        <v>291</v>
       </c>
       <c r="K6" s="9" t="n">
         <v>4229</v>
       </c>
       <c r="L6" s="9" t="n">
-        <v>4994.769862670899</v>
+        <v>5577.999794006348</v>
       </c>
       <c r="M6" s="15" t="n">
-        <v>1.126743878616907</v>
+        <v>1.25017729818074</v>
       </c>
       <c r="N6" s="15" t="n">
-        <v>0.4473595936113658</v>
+        <v>0.4995969363194221</v>
       </c>
       <c r="O6" s="7" t="n"/>
     </row>
@@ -12399,13 +12884,13 @@
         <v>107</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>221.5399932861328</v>
+        <v>225.6849975585938</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>23704.77928161621</v>
+        <v>24148.29473876953</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>0.09865609769600341</v>
+        <v>0.0999819890636468</v>
       </c>
       <c r="H7" s="9" t="n">
         <v>28073.97</v>
@@ -12420,13 +12905,13 @@
         <v>28073.97</v>
       </c>
       <c r="L7" s="9" t="n">
-        <v>-4369.19071838379</v>
+        <v>-3925.67526123047</v>
       </c>
       <c r="M7" s="15" t="n">
-        <v>-0.1556313808978136</v>
+        <v>-0.1398332783439774</v>
       </c>
       <c r="N7" s="15" t="n">
-        <v>-0.1556313808978135</v>
+        <v>-0.1398332783439774</v>
       </c>
       <c r="O7" s="7" t="n"/>
     </row>
@@ -12448,13 +12933,13 @@
         <v>43</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>388.8399963378906</v>
+        <v>396.0132141113281</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>16720.1198425293</v>
+        <v>17028.56820678711</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>0.06958688613281989</v>
+        <v>0.07050394815196401</v>
       </c>
       <c r="H8" s="9" t="n">
         <v>17698.7</v>
@@ -12469,13 +12954,13 @@
         <v>17698.7</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>-915.9701574707033</v>
+        <v>-607.5217932128908</v>
       </c>
       <c r="M8" s="15" t="n">
-        <v>-0.05529107547281454</v>
+        <v>-0.03786333421171556</v>
       </c>
       <c r="N8" s="15" t="n">
-        <v>-0.05175352751731501</v>
+        <v>-0.03432578625621604</v>
       </c>
       <c r="O8" s="7" t="n"/>
     </row>
@@ -12497,13 +12982,13 @@
         <v>500</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>27.05999946594238</v>
+        <v>28.22999954223633</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>13529.99973297119</v>
+        <v>14114.99977111816</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>0.0563100360321894</v>
+        <v>0.05844080370957171</v>
       </c>
       <c r="H9" s="9" t="n">
         <v>12425</v>
@@ -12518,13 +13003,13 @@
         <v>12425</v>
       </c>
       <c r="L9" s="9" t="n">
-        <v>1104.999732971191</v>
+        <v>1689.999771118164</v>
       </c>
       <c r="M9" s="15" t="n">
-        <v>0.08893358011840569</v>
+        <v>0.1360160781584035</v>
       </c>
       <c r="N9" s="15" t="n">
-        <v>0.08893358011840574</v>
+        <v>0.1360160781584036</v>
       </c>
       <c r="O9" s="7" t="n"/>
     </row>
@@ -12546,13 +13031,13 @@
         <v>25</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>234.3999938964844</v>
+        <v>209.9700012207031</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>5859.999847412109</v>
+        <v>5249.250030517578</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>0.02438852986465931</v>
+        <v>0.02173364474887549</v>
       </c>
       <c r="H10" s="9" t="n">
         <v>5210</v>
@@ -12561,19 +13046,19 @@
         <v>0</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="K10" s="9" t="n">
         <v>5210</v>
       </c>
       <c r="L10" s="9" t="n">
-        <v>651.7498474121094</v>
+        <v>42.75003051757812</v>
       </c>
       <c r="M10" s="15" t="n">
-        <v>0.1247600474879288</v>
+        <v>0.007533595108940112</v>
       </c>
       <c r="N10" s="15" t="n">
-        <v>0.1250959400023243</v>
+        <v>0.008205380137730926</v>
       </c>
       <c r="O10" s="7" t="n"/>
     </row>
@@ -12595,13 +13080,13 @@
         <v>430</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>37.09999847412109</v>
+        <v>37.125</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>15952.99934387207</v>
+        <v>15963.75</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>0.06639423396926115</v>
+        <v>0.06609524586232211</v>
       </c>
       <c r="H11" s="9" t="n">
         <v>17180.9</v>
@@ -12616,13 +13101,13 @@
         <v>17180.9</v>
       </c>
       <c r="L11" s="9" t="n">
-        <v>-1087.390656127931</v>
+        <v>-1076.640000000001</v>
       </c>
       <c r="M11" s="15" t="n">
-        <v>-0.0714689367918987</v>
+        <v>-0.07084320379025562</v>
       </c>
       <c r="N11" s="15" t="n">
-        <v>-0.06329066906436397</v>
+        <v>-0.06266493606272087</v>
       </c>
       <c r="O11" s="7" t="n"/>
     </row>
@@ -12644,13 +13129,13 @@
         <v>200</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>23.40999984741211</v>
+        <v>23.61499977111816</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>4681.999969482422</v>
+        <v>4722.999954223633</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>0.01948585308111966</v>
+        <v>0.01955479402910639</v>
       </c>
       <c r="H12" s="9" t="n">
         <v>5947</v>
@@ -12665,13 +13150,13 @@
         <v>5947</v>
       </c>
       <c r="L12" s="9" t="n">
-        <v>-1218.800030517578</v>
+        <v>-1177.800045776367</v>
       </c>
       <c r="M12" s="15" t="n">
-        <v>-0.2127122970434804</v>
+        <v>-0.2058180672231995</v>
       </c>
       <c r="N12" s="15" t="n">
-        <v>-0.2049436742084376</v>
+        <v>-0.1980494443881566</v>
       </c>
       <c r="O12" s="7" t="n"/>
     </row>
@@ -12693,13 +13178,13 @@
         <v>120</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>128.2200012207031</v>
+        <v>125.8949966430664</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>15386.40014648438</v>
+        <v>15107.39959716797</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>0.06403612444595044</v>
+        <v>0.06254966976525959</v>
       </c>
       <c r="H13" s="9" t="n">
         <v>14520</v>
@@ -12714,13 +13199,13 @@
         <v>14520</v>
       </c>
       <c r="L13" s="9" t="n">
-        <v>1070.880146484375</v>
+        <v>791.8795971679683</v>
       </c>
       <c r="M13" s="15" t="n">
-        <v>0.05966943157605888</v>
+        <v>0.04045451771129261</v>
       </c>
       <c r="N13" s="15" t="n">
-        <v>0.07375207620415802</v>
+        <v>0.05453716233939176</v>
       </c>
       <c r="O13" s="7" t="n"/>
     </row>
@@ -12739,19 +13224,19 @@
         </is>
       </c>
       <c r="D14" s="13" t="n">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>141.6000061035156</v>
+        <v>131.5500030517578</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>5522.400238037109</v>
+        <v>7893.000183105469</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>0.02298348577422718</v>
+        <v>0.03267965156643705</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>17927.57</v>
+        <v>20737.43</v>
       </c>
       <c r="I14" s="9" t="n">
         <v>15703.6</v>
@@ -12760,16 +13245,16 @@
         <v>28</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>2223.969999999999</v>
+        <v>5033.83</v>
       </c>
       <c r="L14" s="9" t="n">
-        <v>3326.430238037108</v>
+        <v>2887.170183105467</v>
       </c>
       <c r="M14" s="15" t="n">
-        <v>1.483127127630818</v>
+        <v>0.5679910094511473</v>
       </c>
       <c r="N14" s="15" t="n">
-        <v>0.1855483056564335</v>
+        <v>0.1392250719161182</v>
       </c>
       <c r="O14" s="7" t="n"/>
     </row>
@@ -12791,13 +13276,13 @@
         <v>40</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>352.2000122070312</v>
+        <v>357.4100036621094</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>14088.00048828125</v>
+        <v>14296.40014648438</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>0.0586323599980154</v>
+        <v>0.05919186172597432</v>
       </c>
       <c r="H15" s="9" t="n">
         <v>12988</v>
@@ -12812,13 +13297,13 @@
         <v>12988</v>
       </c>
       <c r="L15" s="9" t="n">
-        <v>1118.76048828125</v>
+        <v>1327.160146484375</v>
       </c>
       <c r="M15" s="15" t="n">
-        <v>0.0846936008839891</v>
+        <v>0.100739155103509</v>
       </c>
       <c r="N15" s="15" t="n">
-        <v>0.086138011108812</v>
+        <v>0.1021835653283319</v>
       </c>
       <c r="O15" s="7" t="n"/>
     </row>
@@ -12840,13 +13325,13 @@
         <v>200</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>84.55000305175781</v>
+        <v>84.36499786376953</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>16910.00061035156</v>
+        <v>16872.99957275391</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>0.07037714430642766</v>
+        <v>0.06985984215463317</v>
       </c>
       <c r="H16" s="9" t="n">
         <v>17734</v>
@@ -12855,19 +13340,19 @@
         <v>0</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>136.57</v>
+        <v>181.1</v>
       </c>
       <c r="K16" s="9" t="n">
         <v>17734</v>
       </c>
       <c r="L16" s="9" t="n">
-        <v>-687.4293896484378</v>
+        <v>-679.9004272460952</v>
       </c>
       <c r="M16" s="15" t="n">
-        <v>-0.04646438421385124</v>
+        <v>-0.04855083045258227</v>
       </c>
       <c r="N16" s="15" t="n">
-        <v>-0.03876335793664361</v>
+        <v>-0.03833880834815018</v>
       </c>
       <c r="O16" s="7" t="n"/>
     </row>
@@ -12889,13 +13374,13 @@
         <v>150</v>
       </c>
       <c r="E17" s="10" t="n">
-        <v>100.4599990844727</v>
+        <v>100.5363006591797</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>15068.9998626709</v>
+        <v>15080.44509887695</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>0.06271514722711061</v>
+        <v>0.06243806915815661</v>
       </c>
       <c r="H17" s="9" t="n">
         <v>16683</v>
@@ -12904,19 +13389,19 @@
         <v>1607.52</v>
       </c>
       <c r="J17" s="9" t="n">
-        <v>93.29000000000001</v>
+        <v>124.34</v>
       </c>
       <c r="K17" s="9" t="n">
         <v>15075.48</v>
       </c>
       <c r="L17" s="9" t="n">
-        <v>86.80986267089975</v>
+        <v>129.3050988769537</v>
       </c>
       <c r="M17" s="15" t="n">
-        <v>-0.0004298461693491978</v>
+        <v>0.0003293493060887112</v>
       </c>
       <c r="N17" s="15" t="n">
-        <v>0.005203492337762977</v>
+        <v>0.007750710236585369</v>
       </c>
       <c r="O17" s="7" t="n"/>
     </row>
@@ -12938,13 +13423,13 @@
         <v>150</v>
       </c>
       <c r="E18" s="10" t="n">
-        <v>49.63999938964844</v>
+        <v>50.9098014831543</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>7445.999908447266</v>
+        <v>7636.470222473145</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>0.03098924844163833</v>
+        <v>0.03161753202566215</v>
       </c>
       <c r="H18" s="9" t="n">
         <v>5769</v>
@@ -12959,13 +13444,13 @@
         <v>5769</v>
       </c>
       <c r="L18" s="9" t="n">
-        <v>1808.059908447266</v>
+        <v>1998.530222473145</v>
       </c>
       <c r="M18" s="15" t="n">
-        <v>0.2906916117953312</v>
+        <v>0.3237077868734866</v>
       </c>
       <c r="N18" s="15" t="n">
-        <v>0.3134095871810134</v>
+        <v>0.3464257622591688</v>
       </c>
       <c r="O18" s="7" t="n"/>
     </row>
@@ -12984,37 +13469,37 @@
         </is>
       </c>
       <c r="D19" s="13" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="E19" s="10" t="n">
-        <v>45.65000152587891</v>
+        <v>54.7400016784668</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>18260.00061035156</v>
+        <v>16422.00050354004</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>0.07599566242496143</v>
+        <v>0.06799255568601716</v>
       </c>
       <c r="H19" s="9" t="n">
         <v>18236.4</v>
       </c>
       <c r="I19" s="9" t="n">
-        <v>0</v>
+        <v>5630</v>
       </c>
       <c r="J19" s="9" t="n">
         <v>39.2</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>18236.4</v>
+        <v>12606.4</v>
       </c>
       <c r="L19" s="9" t="n">
-        <v>62.80061035156177</v>
+        <v>3854.800503540038</v>
       </c>
       <c r="M19" s="15" t="n">
-        <v>0.001294148535432545</v>
+        <v>0.3026716987831607</v>
       </c>
       <c r="N19" s="15" t="n">
-        <v>0.003443695595159229</v>
+        <v>0.2113794665361605</v>
       </c>
       <c r="O19" s="7" t="n"/>
     </row>
@@ -13036,13 +13521,13 @@
         <v>40</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>196.9299926757812</v>
+        <v>209.4550018310547</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>7877.19970703125</v>
+        <v>8378.200073242188</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>0.03278384390908443</v>
+        <v>0.03468854083311675</v>
       </c>
       <c r="H20" s="9" t="n">
         <v>8635</v>
@@ -13057,13 +13542,13 @@
         <v>8635</v>
       </c>
       <c r="L20" s="9" t="n">
-        <v>-757.80029296875</v>
+        <v>-256.7999267578125</v>
       </c>
       <c r="M20" s="15" t="n">
-        <v>-0.08775915378908512</v>
+        <v>-0.02973942405996671</v>
       </c>
       <c r="N20" s="15" t="n">
-        <v>-0.08775915378908512</v>
+        <v>-0.02973942405996671</v>
       </c>
       <c r="O20" s="7" t="n"/>
     </row>
@@ -13085,13 +13570,13 @@
         <v>10</v>
       </c>
       <c r="E21" s="10" t="n">
-        <v>535.3800048828125</v>
+        <v>515.9500122070312</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>5353.800048828125</v>
+        <v>5159.500122070312</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>0.02228179450173911</v>
+        <v>0.02136205021344723</v>
       </c>
       <c r="H21" s="9" t="n">
         <v>5069.8</v>
@@ -13106,13 +13591,13 @@
         <v>5069.8</v>
       </c>
       <c r="L21" s="9" t="n">
-        <v>284.0000488281248</v>
+        <v>89.70012207031232</v>
       </c>
       <c r="M21" s="15" t="n">
-        <v>0.05601799850647458</v>
+        <v>0.01769302971918267</v>
       </c>
       <c r="N21" s="15" t="n">
-        <v>0.05601799850647458</v>
+        <v>0.01769302971918267</v>
       </c>
       <c r="O21" s="7" t="n"/>
     </row>
@@ -13134,16 +13619,16 @@
         <v>38</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>443.4599914550781</v>
+        <v>447.5299987792969</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>16851.47967529297</v>
+        <v>17006.13995361328</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>0.07013358805906453</v>
+        <v>0.07041108770828464</v>
       </c>
       <c r="H22" s="9" t="n">
-        <v>14284.37917736824</v>
+        <v>14284.70668805384</v>
       </c>
       <c r="I22" s="9" t="n">
         <v>0</v>
@@ -13152,67 +13637,18 @@
         <v>51.6</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>14284.37917736824</v>
+        <v>14284.70668805384</v>
       </c>
       <c r="L22" s="9" t="n">
-        <v>2618.700497924729</v>
+        <v>2773.033265559436</v>
       </c>
       <c r="M22" s="15" t="n">
-        <v>0.1797138304751787</v>
+        <v>0.190513765874895</v>
       </c>
       <c r="N22" s="15" t="n">
-        <v>0.1833261680755242</v>
+        <v>0.1941260206538574</v>
       </c>
       <c r="O22" s="7" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>MBGL</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>Mobility Global Inc.</t>
-        </is>
-      </c>
-      <c r="D23" s="13" t="n">
-        <v>38</v>
-      </c>
-      <c r="E23" s="10" t="n">
-        <v>21.20000076293945</v>
-      </c>
-      <c r="F23" s="9" t="n">
-        <v>805.6000289916992</v>
-      </c>
-      <c r="G23" s="14" t="n">
-        <v>0.003352798784578661</v>
-      </c>
-      <c r="H23" s="9" t="n">
-        <v>729.7608226317609</v>
-      </c>
-      <c r="I23" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" s="9" t="n">
-        <v>729.7608226317609</v>
-      </c>
-      <c r="L23" s="9" t="n">
-        <v>75.83920635993832</v>
-      </c>
-      <c r="M23" s="15" t="n">
-        <v>0.1039233732587026</v>
-      </c>
-      <c r="N23" s="15" t="n">
-        <v>0.1039233732587025</v>
-      </c>
-      <c r="O23" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
data: 更新淨值表至 2026-07-17（via Portal）
</commit_message>
<xml_diff>
--- a/assets/data/Yi_Capital_US.xlsx
+++ b/assets/data/Yi_Capital_US.xlsx
@@ -4963,7 +4963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J133"/>
+  <dimension ref="A1:J135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5275,7 +5275,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>153121.44</v>
+        <v>153121.43</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>0</v>
@@ -5284,7 +5284,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>153121.44</v>
+        <v>153121.43</v>
       </c>
       <c r="F9" s="8" t="n">
         <v>1513476.32</v>
@@ -5299,7 +5299,7 @@
         <v>13619.69</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>139501.75</v>
+        <v>139501.74</v>
       </c>
     </row>
     <row r="10">
@@ -5309,7 +5309,7 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>153368.68</v>
+        <v>153368.67</v>
       </c>
       <c r="C10" s="9" t="n">
         <v>0</v>
@@ -5318,7 +5318,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>153368.68</v>
+        <v>153368.67</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>1513476.32</v>
@@ -5333,7 +5333,7 @@
         <v>13619.69</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>139748.99</v>
+        <v>139748.98</v>
       </c>
     </row>
     <row r="11">
@@ -5615,7 +5615,7 @@
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>155929.2</v>
+        <v>155929.19</v>
       </c>
       <c r="C19" s="9" t="n">
         <v>0</v>
@@ -5624,7 +5624,7 @@
         <v>0</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>155929.2</v>
+        <v>155929.19</v>
       </c>
       <c r="F19" s="8" t="n">
         <v>1513476.32</v>
@@ -5639,7 +5639,7 @@
         <v>27249.8</v>
       </c>
       <c r="J19" s="9" t="n">
-        <v>128679.4</v>
+        <v>128679.39</v>
       </c>
     </row>
     <row r="20">
@@ -5649,7 +5649,7 @@
         </is>
       </c>
       <c r="B20" s="9" t="n">
-        <v>205195.02</v>
+        <v>205195.01</v>
       </c>
       <c r="C20" s="9" t="n">
         <v>0</v>
@@ -5658,7 +5658,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>205195.02</v>
+        <v>205195.01</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>2005476.32</v>
@@ -5673,7 +5673,7 @@
         <v>39507.2</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>165687.82</v>
+        <v>165687.81</v>
       </c>
     </row>
     <row r="21">
@@ -5683,7 +5683,7 @@
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>204602.42</v>
+        <v>204602.43</v>
       </c>
       <c r="C21" s="9" t="n">
         <v>0</v>
@@ -5692,7 +5692,7 @@
         <v>0</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>204602.42</v>
+        <v>204602.43</v>
       </c>
       <c r="F21" s="8" t="n">
         <v>2005476.32</v>
@@ -5707,7 +5707,7 @@
         <v>39507.2</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>165095.22</v>
+        <v>165095.23</v>
       </c>
     </row>
     <row r="22">
@@ -5751,7 +5751,7 @@
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>208407.9</v>
+        <v>208407.89</v>
       </c>
       <c r="C23" s="9" t="n">
         <v>0</v>
@@ -5760,7 +5760,7 @@
         <v>0</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>208407.9</v>
+        <v>208407.89</v>
       </c>
       <c r="F23" s="8" t="n">
         <v>2054841.55</v>
@@ -5775,7 +5775,7 @@
         <v>13000.1</v>
       </c>
       <c r="J23" s="9" t="n">
-        <v>195407.8</v>
+        <v>195407.79</v>
       </c>
     </row>
     <row r="24">
@@ -5785,7 +5785,7 @@
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>206929.2</v>
+        <v>206929.19</v>
       </c>
       <c r="C24" s="9" t="n">
         <v>0</v>
@@ -5794,7 +5794,7 @@
         <v>0</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>206929.2</v>
+        <v>206929.19</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>2054841.55</v>
@@ -5809,7 +5809,7 @@
         <v>13000.1</v>
       </c>
       <c r="J24" s="9" t="n">
-        <v>193929.1</v>
+        <v>193929.09</v>
       </c>
     </row>
     <row r="25">
@@ -5921,7 +5921,7 @@
         </is>
       </c>
       <c r="B28" s="9" t="n">
-        <v>214482.66</v>
+        <v>214482.65</v>
       </c>
       <c r="C28" s="9" t="n">
         <v>0</v>
@@ -5930,7 +5930,7 @@
         <v>0</v>
       </c>
       <c r="E28" s="9" t="n">
-        <v>214482.66</v>
+        <v>214482.65</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>2107072.57</v>
@@ -5945,7 +5945,7 @@
         <v>0</v>
       </c>
       <c r="J28" s="9" t="n">
-        <v>214482.66</v>
+        <v>214482.65</v>
       </c>
     </row>
     <row r="29">
@@ -6091,7 +6091,7 @@
         </is>
       </c>
       <c r="B33" s="9" t="n">
-        <v>214364.04</v>
+        <v>214364.05</v>
       </c>
       <c r="C33" s="9" t="n">
         <v>0</v>
@@ -6100,7 +6100,7 @@
         <v>0</v>
       </c>
       <c r="E33" s="9" t="n">
-        <v>214364.04</v>
+        <v>214364.05</v>
       </c>
       <c r="F33" s="8" t="n">
         <v>2107072.57</v>
@@ -6115,7 +6115,7 @@
         <v>0</v>
       </c>
       <c r="J33" s="9" t="n">
-        <v>214364.04</v>
+        <v>214364.05</v>
       </c>
     </row>
     <row r="34">
@@ -6295,7 +6295,7 @@
         </is>
       </c>
       <c r="B39" s="9" t="n">
-        <v>217434.09</v>
+        <v>217434.08</v>
       </c>
       <c r="C39" s="9" t="n">
         <v>0</v>
@@ -6304,13 +6304,13 @@
         <v>0</v>
       </c>
       <c r="E39" s="9" t="n">
-        <v>217434.09</v>
+        <v>217434.08</v>
       </c>
       <c r="F39" s="8" t="n">
         <v>2107072.57</v>
       </c>
       <c r="G39" s="16" t="n">
-        <v>0.103193</v>
+        <v>0.103192</v>
       </c>
       <c r="H39" s="9" t="n">
         <v>-0</v>
@@ -6319,7 +6319,7 @@
         <v>0</v>
       </c>
       <c r="J39" s="9" t="n">
-        <v>217434.09</v>
+        <v>217434.08</v>
       </c>
     </row>
     <row r="40">
@@ -6737,7 +6737,7 @@
         </is>
       </c>
       <c r="B52" s="9" t="n">
-        <v>215143.4</v>
+        <v>215143.41</v>
       </c>
       <c r="C52" s="9" t="n">
         <v>0</v>
@@ -6746,7 +6746,7 @@
         <v>0</v>
       </c>
       <c r="E52" s="9" t="n">
-        <v>215143.4</v>
+        <v>215143.41</v>
       </c>
       <c r="F52" s="8" t="n">
         <v>2107072.57</v>
@@ -6761,7 +6761,7 @@
         <v>-12742.44</v>
       </c>
       <c r="J52" s="9" t="n">
-        <v>227885.84</v>
+        <v>227885.85</v>
       </c>
     </row>
     <row r="53">
@@ -6839,7 +6839,7 @@
         </is>
       </c>
       <c r="B55" s="9" t="n">
-        <v>213029.51</v>
+        <v>213029.52</v>
       </c>
       <c r="C55" s="9" t="n">
         <v>0</v>
@@ -6848,7 +6848,7 @@
         <v>0</v>
       </c>
       <c r="E55" s="9" t="n">
-        <v>213029.51</v>
+        <v>213029.52</v>
       </c>
       <c r="F55" s="8" t="n">
         <v>2107072.57</v>
@@ -6863,7 +6863,7 @@
         <v>-12742.44</v>
       </c>
       <c r="J55" s="9" t="n">
-        <v>225771.95</v>
+        <v>225771.96</v>
       </c>
     </row>
     <row r="56">
@@ -6873,7 +6873,7 @@
         </is>
       </c>
       <c r="B56" s="9" t="n">
-        <v>210102.87</v>
+        <v>210102.88</v>
       </c>
       <c r="C56" s="9" t="n">
         <v>0</v>
@@ -6882,7 +6882,7 @@
         <v>0</v>
       </c>
       <c r="E56" s="9" t="n">
-        <v>210102.87</v>
+        <v>210102.88</v>
       </c>
       <c r="F56" s="8" t="n">
         <v>2107072.57</v>
@@ -6897,7 +6897,7 @@
         <v>-12742.44</v>
       </c>
       <c r="J56" s="9" t="n">
-        <v>222845.31</v>
+        <v>222845.32</v>
       </c>
     </row>
     <row r="57">
@@ -7009,7 +7009,7 @@
         </is>
       </c>
       <c r="B60" s="9" t="n">
-        <v>210662.18</v>
+        <v>210662.17</v>
       </c>
       <c r="C60" s="9" t="n">
         <v>0</v>
@@ -7018,7 +7018,7 @@
         <v>0</v>
       </c>
       <c r="E60" s="9" t="n">
-        <v>210662.18</v>
+        <v>210662.17</v>
       </c>
       <c r="F60" s="8" t="n">
         <v>2107072.57</v>
@@ -7033,7 +7033,7 @@
         <v>-5792.88</v>
       </c>
       <c r="J60" s="9" t="n">
-        <v>216455.06</v>
+        <v>216455.05</v>
       </c>
     </row>
     <row r="61">
@@ -7247,7 +7247,7 @@
         </is>
       </c>
       <c r="B67" s="9" t="n">
-        <v>213604.99</v>
+        <v>213605</v>
       </c>
       <c r="C67" s="9" t="n">
         <v>0</v>
@@ -7256,7 +7256,7 @@
         <v>0</v>
       </c>
       <c r="E67" s="9" t="n">
-        <v>213604.99</v>
+        <v>213605</v>
       </c>
       <c r="F67" s="8" t="n">
         <v>2107072.57</v>
@@ -7271,7 +7271,7 @@
         <v>-5521.95</v>
       </c>
       <c r="J67" s="9" t="n">
-        <v>219126.94</v>
+        <v>219126.95</v>
       </c>
     </row>
     <row r="68">
@@ -7281,7 +7281,7 @@
         </is>
       </c>
       <c r="B68" s="9" t="n">
-        <v>211847.57</v>
+        <v>211847.56</v>
       </c>
       <c r="C68" s="9" t="n">
         <v>0</v>
@@ -7290,7 +7290,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="9" t="n">
-        <v>211847.57</v>
+        <v>211847.56</v>
       </c>
       <c r="F68" s="8" t="n">
         <v>2107072.57</v>
@@ -7305,7 +7305,7 @@
         <v>-5521.95</v>
       </c>
       <c r="J68" s="9" t="n">
-        <v>217369.52</v>
+        <v>217369.51</v>
       </c>
     </row>
     <row r="69">
@@ -7723,7 +7723,7 @@
         </is>
       </c>
       <c r="B81" s="9" t="n">
-        <v>223631.68</v>
+        <v>223631.67</v>
       </c>
       <c r="C81" s="9" t="n">
         <v>0</v>
@@ -7732,7 +7732,7 @@
         <v>0</v>
       </c>
       <c r="E81" s="9" t="n">
-        <v>223631.68</v>
+        <v>223631.67</v>
       </c>
       <c r="F81" s="8" t="n">
         <v>2107072.57</v>
@@ -7747,7 +7747,7 @@
         <v>-3671.5</v>
       </c>
       <c r="J81" s="9" t="n">
-        <v>227303.18</v>
+        <v>227303.17</v>
       </c>
     </row>
     <row r="82">
@@ -8267,7 +8267,7 @@
         </is>
       </c>
       <c r="B97" s="9" t="n">
-        <v>220861.6</v>
+        <v>220861.61</v>
       </c>
       <c r="C97" s="9" t="n">
         <v>0</v>
@@ -8276,7 +8276,7 @@
         <v>0</v>
       </c>
       <c r="E97" s="9" t="n">
-        <v>220861.6</v>
+        <v>220861.61</v>
       </c>
       <c r="F97" s="8" t="n">
         <v>2107072.57</v>
@@ -8291,7 +8291,7 @@
         <v>-4903.56</v>
       </c>
       <c r="J97" s="9" t="n">
-        <v>225765.16</v>
+        <v>225765.17</v>
       </c>
     </row>
     <row r="98">
@@ -8403,7 +8403,7 @@
         </is>
       </c>
       <c r="B101" s="9" t="n">
-        <v>220806.2</v>
+        <v>220806.21</v>
       </c>
       <c r="C101" s="9" t="n">
         <v>0</v>
@@ -8412,7 +8412,7 @@
         <v>0</v>
       </c>
       <c r="E101" s="9" t="n">
-        <v>220806.2</v>
+        <v>220806.21</v>
       </c>
       <c r="F101" s="8" t="n">
         <v>2107072.57</v>
@@ -8427,7 +8427,7 @@
         <v>-2876.06</v>
       </c>
       <c r="J101" s="9" t="n">
-        <v>223682.26</v>
+        <v>223682.27</v>
       </c>
     </row>
     <row r="102">
@@ -9491,7 +9491,7 @@
         </is>
       </c>
       <c r="B133" s="9" t="n">
-        <v>228717</v>
+        <v>228347.57</v>
       </c>
       <c r="C133" s="9" t="n">
         <v>0</v>
@@ -9500,13 +9500,13 @@
         <v>0</v>
       </c>
       <c r="E133" s="9" t="n">
-        <v>228717</v>
+        <v>228347.57</v>
       </c>
       <c r="F133" s="8" t="n">
         <v>2107072.57</v>
       </c>
       <c r="G133" s="16" t="n">
-        <v>0.108547</v>
+        <v>0.108372</v>
       </c>
       <c r="H133" s="9" t="n">
         <v>-0</v>
@@ -9515,7 +9515,75 @@
         <v>-12809.08</v>
       </c>
       <c r="J133" s="9" t="n">
-        <v>241526.08</v>
+        <v>241156.65</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B134" s="9" t="n">
+        <v>231260.73</v>
+      </c>
+      <c r="C134" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D134" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E134" s="9" t="n">
+        <v>231260.73</v>
+      </c>
+      <c r="F134" s="8" t="n">
+        <v>2107072.57</v>
+      </c>
+      <c r="G134" s="16" t="n">
+        <v>0.109755</v>
+      </c>
+      <c r="H134" s="9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I134" s="9" t="n">
+        <v>-12809.08</v>
+      </c>
+      <c r="J134" s="9" t="n">
+        <v>244069.81</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B135" s="9" t="n">
+        <v>231260.73</v>
+      </c>
+      <c r="C135" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D135" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E135" s="9" t="n">
+        <v>231260.73</v>
+      </c>
+      <c r="F135" s="8" t="n">
+        <v>2107072.57</v>
+      </c>
+      <c r="G135" s="16" t="n">
+        <v>0.109755</v>
+      </c>
+      <c r="H135" s="9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I135" s="9" t="n">
+        <v>-12809.08</v>
+      </c>
+      <c r="J135" s="9" t="n">
+        <v>244069.81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deploy v8.1 — US, HK and A fund sources
</commit_message>
<xml_diff>
--- a/assets/data/Yi_Capital_US.xlsx
+++ b/assets/data/Yi_Capital_US.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2149,7 +2149,7 @@
       </c>
       <c r="E55" s="2" t="n"/>
       <c r="F55" s="4" t="n">
-        <v>1388</v>
+        <v>2809.86</v>
       </c>
       <c r="G55" s="2" t="n"/>
       <c r="H55" s="2" t="n"/>
@@ -2234,6 +2234,39 @@
         <v>138.8</v>
       </c>
       <c r="I57" s="7" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Oracle Corporation</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="F58" s="9" t="n">
+        <v>1421.86</v>
+      </c>
+      <c r="G58" s="10" t="n">
+        <v>129.26</v>
+      </c>
+      <c r="H58" s="10" t="n">
+        <v>129.26</v>
+      </c>
+      <c r="I58" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -2260,7 +2293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F103"/>
+  <dimension ref="A1:F110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4706,12 +4739,12 @@
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B102" s="7" t="inlineStr">
         <is>
-          <t>ETF Stock Buy Record</t>
+          <t>ETF Stock Dividend Record</t>
         </is>
       </c>
       <c r="C102" s="7" t="n">
@@ -4721,10 +4754,10 @@
         <v>-16538.54</v>
       </c>
       <c r="E102" s="9" t="n">
-        <v>-1388</v>
+        <v>61.23</v>
       </c>
       <c r="F102" s="9" t="n">
-        <v>-17926.54</v>
+        <v>-16477.31</v>
       </c>
     </row>
     <row r="103">
@@ -4735,20 +4768,188 @@
       </c>
       <c r="B103" s="7" t="inlineStr">
         <is>
-          <t>ETF Stock Sell Record</t>
+          <t>ETF Stock Buy Record</t>
         </is>
       </c>
       <c r="C103" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D103" s="9" t="n">
-        <v>-17926.54</v>
+        <v>-16477.31</v>
       </c>
       <c r="E103" s="9" t="n">
+        <v>-1388</v>
+      </c>
+      <c r="F103" s="9" t="n">
+        <v>-17865.31</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B104" s="7" t="inlineStr">
+        <is>
+          <t>ETF Stock Sell Record</t>
+        </is>
+      </c>
+      <c r="C104" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D104" s="9" t="n">
+        <v>-17865.31</v>
+      </c>
+      <c r="E104" s="9" t="n">
         <v>406.8</v>
       </c>
-      <c r="F103" s="9" t="n">
-        <v>-17519.74</v>
+      <c r="F104" s="9" t="n">
+        <v>-17458.51</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B105" s="7" t="inlineStr">
+        <is>
+          <t>ETF Stock Sell Record</t>
+        </is>
+      </c>
+      <c r="C105" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D105" s="9" t="n">
+        <v>-17458.51</v>
+      </c>
+      <c r="E105" s="9" t="n">
+        <v>363.96</v>
+      </c>
+      <c r="F105" s="9" t="n">
+        <v>-17094.55</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B106" s="7" t="inlineStr">
+        <is>
+          <t>ETF Stock Dividend Record</t>
+        </is>
+      </c>
+      <c r="C106" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D106" s="9" t="n">
+        <v>-17094.55</v>
+      </c>
+      <c r="E106" s="9" t="n">
+        <v>44.53</v>
+      </c>
+      <c r="F106" s="9" t="n">
+        <v>-17050.02</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B107" s="7" t="inlineStr">
+        <is>
+          <t>ETF Stock Dividend Record</t>
+        </is>
+      </c>
+      <c r="C107" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D107" s="9" t="n">
+        <v>-17050.02</v>
+      </c>
+      <c r="E107" s="9" t="n">
+        <v>31.05</v>
+      </c>
+      <c r="F107" s="9" t="n">
+        <v>-17018.97</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B108" s="7" t="inlineStr">
+        <is>
+          <t>ETF Stock Dividend Record</t>
+        </is>
+      </c>
+      <c r="C108" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D108" s="9" t="n">
+        <v>-17018.97</v>
+      </c>
+      <c r="E108" s="9" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="F108" s="9" t="n">
+        <v>-17017.22</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B109" s="7" t="inlineStr">
+        <is>
+          <t>ETF Stock Buy Record</t>
+        </is>
+      </c>
+      <c r="C109" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D109" s="9" t="n">
+        <v>-17017.22</v>
+      </c>
+      <c r="E109" s="9" t="n">
+        <v>-1421.86</v>
+      </c>
+      <c r="F109" s="9" t="n">
+        <v>-18439.08</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B110" s="7" t="inlineStr">
+        <is>
+          <t>ETF Stock Sell Record</t>
+        </is>
+      </c>
+      <c r="C110" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D110" s="9" t="n">
+        <v>-18439.08</v>
+      </c>
+      <c r="E110" s="9" t="n">
+        <v>5630</v>
+      </c>
+      <c r="F110" s="9" t="n">
+        <v>-12809.08</v>
       </c>
     </row>
   </sheetData>
@@ -4762,7 +4963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J132"/>
+  <dimension ref="A1:J135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5074,7 +5275,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>153121.43</v>
+        <v>153121.44</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>0</v>
@@ -5083,7 +5284,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>153121.43</v>
+        <v>153121.44</v>
       </c>
       <c r="F9" s="8" t="n">
         <v>1513476.32</v>
@@ -5098,7 +5299,7 @@
         <v>13619.69</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>139501.74</v>
+        <v>139501.75</v>
       </c>
     </row>
     <row r="10">
@@ -5380,7 +5581,7 @@
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>156915.99</v>
+        <v>156916</v>
       </c>
       <c r="C18" s="9" t="n">
         <v>0</v>
@@ -5389,7 +5590,7 @@
         <v>0</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>156915.99</v>
+        <v>156916</v>
       </c>
       <c r="F18" s="8" t="n">
         <v>1513476.32</v>
@@ -5404,7 +5605,7 @@
         <v>13739.39</v>
       </c>
       <c r="J18" s="9" t="n">
-        <v>143176.6</v>
+        <v>143176.61</v>
       </c>
     </row>
     <row r="19">
@@ -5448,7 +5649,7 @@
         </is>
       </c>
       <c r="B20" s="9" t="n">
-        <v>205195.01</v>
+        <v>205195.02</v>
       </c>
       <c r="C20" s="9" t="n">
         <v>0</v>
@@ -5457,7 +5658,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>205195.01</v>
+        <v>205195.02</v>
       </c>
       <c r="F20" s="8" t="n">
         <v>2005476.32</v>
@@ -5472,7 +5673,7 @@
         <v>39507.2</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>165687.81</v>
+        <v>165687.82</v>
       </c>
     </row>
     <row r="21">
@@ -5550,7 +5751,7 @@
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>208407.89</v>
+        <v>208407.9</v>
       </c>
       <c r="C23" s="9" t="n">
         <v>0</v>
@@ -5559,7 +5760,7 @@
         <v>0</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>208407.89</v>
+        <v>208407.9</v>
       </c>
       <c r="F23" s="8" t="n">
         <v>2054841.55</v>
@@ -5574,7 +5775,7 @@
         <v>13000.1</v>
       </c>
       <c r="J23" s="9" t="n">
-        <v>195407.79</v>
+        <v>195407.8</v>
       </c>
     </row>
     <row r="24">
@@ -5584,7 +5785,7 @@
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>206929.19</v>
+        <v>206929.2</v>
       </c>
       <c r="C24" s="9" t="n">
         <v>0</v>
@@ -5593,7 +5794,7 @@
         <v>0</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>206929.19</v>
+        <v>206929.2</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>2054841.55</v>
@@ -5608,7 +5809,7 @@
         <v>13000.1</v>
       </c>
       <c r="J24" s="9" t="n">
-        <v>193929.09</v>
+        <v>193929.1</v>
       </c>
     </row>
     <row r="25">
@@ -5686,7 +5887,7 @@
         </is>
       </c>
       <c r="B27" s="9" t="n">
-        <v>215332.61</v>
+        <v>215332.6</v>
       </c>
       <c r="C27" s="9" t="n">
         <v>0</v>
@@ -5695,7 +5896,7 @@
         <v>0</v>
       </c>
       <c r="E27" s="9" t="n">
-        <v>215332.61</v>
+        <v>215332.6</v>
       </c>
       <c r="F27" s="8" t="n">
         <v>2107072.57</v>
@@ -5710,7 +5911,7 @@
         <v>0</v>
       </c>
       <c r="J27" s="9" t="n">
-        <v>215332.61</v>
+        <v>215332.6</v>
       </c>
     </row>
     <row r="28">
@@ -5890,7 +6091,7 @@
         </is>
       </c>
       <c r="B33" s="9" t="n">
-        <v>214364.04</v>
+        <v>214364.05</v>
       </c>
       <c r="C33" s="9" t="n">
         <v>0</v>
@@ -5899,7 +6100,7 @@
         <v>0</v>
       </c>
       <c r="E33" s="9" t="n">
-        <v>214364.04</v>
+        <v>214364.05</v>
       </c>
       <c r="F33" s="8" t="n">
         <v>2107072.57</v>
@@ -5914,7 +6115,7 @@
         <v>0</v>
       </c>
       <c r="J33" s="9" t="n">
-        <v>214364.04</v>
+        <v>214364.05</v>
       </c>
     </row>
     <row r="34">
@@ -6570,7 +6771,7 @@
         </is>
       </c>
       <c r="B53" s="9" t="n">
-        <v>214364.98</v>
+        <v>214364.99</v>
       </c>
       <c r="C53" s="9" t="n">
         <v>0</v>
@@ -6579,7 +6780,7 @@
         <v>0</v>
       </c>
       <c r="E53" s="9" t="n">
-        <v>214364.98</v>
+        <v>214364.99</v>
       </c>
       <c r="F53" s="8" t="n">
         <v>2107072.57</v>
@@ -6594,7 +6795,7 @@
         <v>-12742.44</v>
       </c>
       <c r="J53" s="9" t="n">
-        <v>227107.42</v>
+        <v>227107.43</v>
       </c>
     </row>
     <row r="54">
@@ -6638,7 +6839,7 @@
         </is>
       </c>
       <c r="B55" s="9" t="n">
-        <v>213029.51</v>
+        <v>213029.52</v>
       </c>
       <c r="C55" s="9" t="n">
         <v>0</v>
@@ -6647,7 +6848,7 @@
         <v>0</v>
       </c>
       <c r="E55" s="9" t="n">
-        <v>213029.51</v>
+        <v>213029.52</v>
       </c>
       <c r="F55" s="8" t="n">
         <v>2107072.57</v>
@@ -6662,7 +6863,7 @@
         <v>-12742.44</v>
       </c>
       <c r="J55" s="9" t="n">
-        <v>225771.95</v>
+        <v>225771.96</v>
       </c>
     </row>
     <row r="56">
@@ -6876,7 +7077,7 @@
         </is>
       </c>
       <c r="B62" s="9" t="n">
-        <v>212156.27</v>
+        <v>212156.26</v>
       </c>
       <c r="C62" s="9" t="n">
         <v>0</v>
@@ -6885,7 +7086,7 @@
         <v>0</v>
       </c>
       <c r="E62" s="9" t="n">
-        <v>212156.27</v>
+        <v>212156.26</v>
       </c>
       <c r="F62" s="8" t="n">
         <v>2107072.57</v>
@@ -6900,7 +7101,7 @@
         <v>-5732.01</v>
       </c>
       <c r="J62" s="9" t="n">
-        <v>217888.28</v>
+        <v>217888.27</v>
       </c>
     </row>
     <row r="63">
@@ -7318,7 +7519,7 @@
         </is>
       </c>
       <c r="B75" s="9" t="n">
-        <v>224658.3</v>
+        <v>224658.29</v>
       </c>
       <c r="C75" s="9" t="n">
         <v>0</v>
@@ -7327,7 +7528,7 @@
         <v>0</v>
       </c>
       <c r="E75" s="9" t="n">
-        <v>224658.3</v>
+        <v>224658.29</v>
       </c>
       <c r="F75" s="8" t="n">
         <v>2107072.57</v>
@@ -7342,7 +7543,7 @@
         <v>-3745.7</v>
       </c>
       <c r="J75" s="9" t="n">
-        <v>228404</v>
+        <v>228403.99</v>
       </c>
     </row>
     <row r="76">
@@ -8066,7 +8267,7 @@
         </is>
       </c>
       <c r="B97" s="9" t="n">
-        <v>220861.6</v>
+        <v>220861.61</v>
       </c>
       <c r="C97" s="9" t="n">
         <v>0</v>
@@ -8075,7 +8276,7 @@
         <v>0</v>
       </c>
       <c r="E97" s="9" t="n">
-        <v>220861.6</v>
+        <v>220861.61</v>
       </c>
       <c r="F97" s="8" t="n">
         <v>2107072.57</v>
@@ -8090,7 +8291,7 @@
         <v>-4903.56</v>
       </c>
       <c r="J97" s="9" t="n">
-        <v>225765.16</v>
+        <v>225765.17</v>
       </c>
     </row>
     <row r="98">
@@ -9052,7 +9253,7 @@
         </is>
       </c>
       <c r="B126" s="9" t="n">
-        <v>221887.09</v>
+        <v>221948.32</v>
       </c>
       <c r="C126" s="9" t="n">
         <v>0</v>
@@ -9061,19 +9262,19 @@
         <v>0</v>
       </c>
       <c r="E126" s="9" t="n">
-        <v>221887.09</v>
+        <v>221948.32</v>
       </c>
       <c r="F126" s="8" t="n">
         <v>2107072.57</v>
       </c>
       <c r="G126" s="16" t="n">
-        <v>0.105306</v>
+        <v>0.105335</v>
       </c>
       <c r="H126" s="9" t="n">
         <v>-0</v>
       </c>
       <c r="I126" s="9" t="n">
-        <v>-16538.54</v>
+        <v>-16477.31</v>
       </c>
       <c r="J126" s="9" t="n">
         <v>238425.63</v>
@@ -9086,7 +9287,7 @@
         </is>
       </c>
       <c r="B127" s="9" t="n">
-        <v>223453.64</v>
+        <v>223514.87</v>
       </c>
       <c r="C127" s="9" t="n">
         <v>0</v>
@@ -9095,19 +9296,19 @@
         <v>0</v>
       </c>
       <c r="E127" s="9" t="n">
-        <v>223453.64</v>
+        <v>223514.87</v>
       </c>
       <c r="F127" s="8" t="n">
         <v>2107072.57</v>
       </c>
       <c r="G127" s="16" t="n">
-        <v>0.106049</v>
+        <v>0.106078</v>
       </c>
       <c r="H127" s="9" t="n">
         <v>-0</v>
       </c>
       <c r="I127" s="9" t="n">
-        <v>-17519.74</v>
+        <v>-17458.51</v>
       </c>
       <c r="J127" s="9" t="n">
         <v>240973.38</v>
@@ -9120,7 +9321,7 @@
         </is>
       </c>
       <c r="B128" s="9" t="n">
-        <v>221746.61</v>
+        <v>221829.33</v>
       </c>
       <c r="C128" s="9" t="n">
         <v>0</v>
@@ -9129,22 +9330,22 @@
         <v>0</v>
       </c>
       <c r="E128" s="9" t="n">
-        <v>221746.61</v>
+        <v>221829.33</v>
       </c>
       <c r="F128" s="8" t="n">
         <v>2107072.57</v>
       </c>
       <c r="G128" s="16" t="n">
-        <v>0.105239</v>
+        <v>0.105278</v>
       </c>
       <c r="H128" s="9" t="n">
         <v>-0</v>
       </c>
       <c r="I128" s="9" t="n">
-        <v>-17519.74</v>
+        <v>-17050.02</v>
       </c>
       <c r="J128" s="9" t="n">
-        <v>239266.35</v>
+        <v>238879.35</v>
       </c>
     </row>
     <row r="129">
@@ -9154,7 +9355,7 @@
         </is>
       </c>
       <c r="B129" s="9" t="n">
-        <v>222272.13</v>
+        <v>222341.17</v>
       </c>
       <c r="C129" s="9" t="n">
         <v>0</v>
@@ -9163,22 +9364,22 @@
         <v>0</v>
       </c>
       <c r="E129" s="9" t="n">
-        <v>222272.13</v>
+        <v>222341.17</v>
       </c>
       <c r="F129" s="8" t="n">
         <v>2107072.57</v>
       </c>
       <c r="G129" s="16" t="n">
-        <v>0.105489</v>
+        <v>0.105521</v>
       </c>
       <c r="H129" s="9" t="n">
         <v>-0</v>
       </c>
       <c r="I129" s="9" t="n">
-        <v>-17519.74</v>
+        <v>-17050.02</v>
       </c>
       <c r="J129" s="9" t="n">
-        <v>239791.87</v>
+        <v>239391.19</v>
       </c>
     </row>
     <row r="130">
@@ -9188,7 +9389,7 @@
         </is>
       </c>
       <c r="B130" s="9" t="n">
-        <v>223492</v>
+        <v>223618.37</v>
       </c>
       <c r="C130" s="9" t="n">
         <v>0</v>
@@ -9197,22 +9398,22 @@
         <v>0</v>
       </c>
       <c r="E130" s="9" t="n">
-        <v>223492</v>
+        <v>223618.37</v>
       </c>
       <c r="F130" s="8" t="n">
         <v>2107072.57</v>
       </c>
       <c r="G130" s="16" t="n">
-        <v>0.106068</v>
+        <v>0.106128</v>
       </c>
       <c r="H130" s="9" t="n">
         <v>-0</v>
       </c>
       <c r="I130" s="9" t="n">
-        <v>-17519.74</v>
+        <v>-17018.97</v>
       </c>
       <c r="J130" s="9" t="n">
-        <v>241011.74</v>
+        <v>240637.34</v>
       </c>
     </row>
     <row r="131">
@@ -9222,7 +9423,7 @@
         </is>
       </c>
       <c r="B131" s="9" t="n">
-        <v>225633.76</v>
+        <v>225771.6</v>
       </c>
       <c r="C131" s="9" t="n">
         <v>0</v>
@@ -9231,22 +9432,22 @@
         <v>0</v>
       </c>
       <c r="E131" s="9" t="n">
-        <v>225633.76</v>
+        <v>225771.6</v>
       </c>
       <c r="F131" s="8" t="n">
         <v>2107072.57</v>
       </c>
       <c r="G131" s="16" t="n">
-        <v>0.107084</v>
+        <v>0.107149</v>
       </c>
       <c r="H131" s="9" t="n">
         <v>-0</v>
       </c>
       <c r="I131" s="9" t="n">
-        <v>-17519.74</v>
+        <v>-17017.22</v>
       </c>
       <c r="J131" s="9" t="n">
-        <v>243153.5</v>
+        <v>242788.82</v>
       </c>
     </row>
     <row r="132">
@@ -9256,7 +9457,7 @@
         </is>
       </c>
       <c r="B132" s="9" t="n">
-        <v>225633.76</v>
+        <v>223868.53</v>
       </c>
       <c r="C132" s="9" t="n">
         <v>0</v>
@@ -9265,22 +9466,124 @@
         <v>0</v>
       </c>
       <c r="E132" s="9" t="n">
-        <v>225633.76</v>
+        <v>223868.53</v>
       </c>
       <c r="F132" s="8" t="n">
         <v>2107072.57</v>
       </c>
       <c r="G132" s="16" t="n">
-        <v>0.107084</v>
+        <v>0.106246</v>
       </c>
       <c r="H132" s="9" t="n">
         <v>-0</v>
       </c>
       <c r="I132" s="9" t="n">
-        <v>-17519.74</v>
+        <v>-18439.08</v>
       </c>
       <c r="J132" s="9" t="n">
-        <v>243153.5</v>
+        <v>242307.61</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B133" s="9" t="n">
+        <v>228347.57</v>
+      </c>
+      <c r="C133" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D133" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E133" s="9" t="n">
+        <v>228347.57</v>
+      </c>
+      <c r="F133" s="8" t="n">
+        <v>2107072.57</v>
+      </c>
+      <c r="G133" s="16" t="n">
+        <v>0.108372</v>
+      </c>
+      <c r="H133" s="9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I133" s="9" t="n">
+        <v>-12809.08</v>
+      </c>
+      <c r="J133" s="9" t="n">
+        <v>241156.65</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B134" s="9" t="n">
+        <v>231260.73</v>
+      </c>
+      <c r="C134" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D134" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E134" s="9" t="n">
+        <v>231260.73</v>
+      </c>
+      <c r="F134" s="8" t="n">
+        <v>2107072.57</v>
+      </c>
+      <c r="G134" s="16" t="n">
+        <v>0.109755</v>
+      </c>
+      <c r="H134" s="9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I134" s="9" t="n">
+        <v>-12809.08</v>
+      </c>
+      <c r="J134" s="9" t="n">
+        <v>244069.81</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B135" s="9" t="n">
+        <v>230555.13</v>
+      </c>
+      <c r="C135" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D135" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E135" s="9" t="n">
+        <v>230555.13</v>
+      </c>
+      <c r="F135" s="8" t="n">
+        <v>2107072.57</v>
+      </c>
+      <c r="G135" s="16" t="n">
+        <v>0.10942</v>
+      </c>
+      <c r="H135" s="9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I135" s="9" t="n">
+        <v>-12809.08</v>
+      </c>
+      <c r="J135" s="9" t="n">
+        <v>243364.21</v>
       </c>
     </row>
   </sheetData>
@@ -9294,7 +9597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10424,7 +10727,7 @@
       </c>
       <c r="E40" s="2" t="n"/>
       <c r="F40" s="4" t="n">
-        <v>406.8</v>
+        <v>6400.76</v>
       </c>
       <c r="G40" s="2" t="n"/>
       <c r="H40" s="2" t="n"/>
@@ -10509,6 +10812,72 @@
         <v>20.34</v>
       </c>
       <c r="I42" s="7" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>MBGL</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>Mobility Global Inc.</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="F43" s="9" t="n">
+        <v>363.96</v>
+      </c>
+      <c r="G43" s="10" t="n">
+        <v>20.22</v>
+      </c>
+      <c r="H43" s="10" t="n">
+        <v>20.22</v>
+      </c>
+      <c r="I43" s="7" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>PayPal Holdings, Inc.</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="F44" s="9" t="n">
+        <v>5630</v>
+      </c>
+      <c r="G44" s="10" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="H44" s="10" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="I44" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -10537,7 +10906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -11882,11 +12251,195 @@
       </c>
       <c r="H49" s="7" t="n"/>
     </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>2026/07/01-2026/07/31</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n"/>
+      <c r="C51" s="2" t="n"/>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Total Dividend Amount:</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="4" t="n">
+        <v>138.56</v>
+      </c>
+      <c r="G51" s="2" t="n"/>
+      <c r="H51" s="2" t="n"/>
+    </row>
+    <row r="52" ht="28" customHeight="1">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Trade No.</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Execution Date</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Stock/ETF Name</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>Amount (USD)</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>Div Per Share (USD)</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>PBR-A</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Petrobras (Preferred ADR)</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="F53" s="9" t="n">
+        <v>61.23</v>
+      </c>
+      <c r="G53" s="10" t="n">
+        <v>0.10205</v>
+      </c>
+      <c r="H53" s="7" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>TLT</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>iShares 20+ Year Treasury Bond ETF</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="F54" s="9" t="n">
+        <v>44.53</v>
+      </c>
+      <c r="G54" s="10" t="n">
+        <v>0.22265</v>
+      </c>
+      <c r="H54" s="7" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>SGOV</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>iShares 0-3 Month Treasury Bond ETF</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="F55" s="9" t="n">
+        <v>31.05</v>
+      </c>
+      <c r="G55" s="10" t="n">
+        <v>0.207</v>
+      </c>
+      <c r="H55" s="7" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>PGR</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>The Progressive Corporation</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="F56" s="9" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="G56" s="10" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="H56" s="7" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="14">
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="D39:E39"/>
     <mergeCell ref="D1:E1"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="D51:E51"/>
     <mergeCell ref="D23:E23"/>
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="D32:E32"/>
@@ -12057,7 +12610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -12085,7 +12638,7 @@
       </c>
       <c r="B1" s="12" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="C1" s="2" t="n"/>
@@ -12103,7 +12656,7 @@
       </c>
       <c r="L1" s="2" t="n"/>
       <c r="M1" s="4" t="n">
-        <v>240276.88</v>
+        <v>243363.9</v>
       </c>
       <c r="N1" s="2" t="n"/>
       <c r="O1" s="2" t="n"/>
@@ -12203,13 +12756,13 @@
         <v>20</v>
       </c>
       <c r="E3" s="10" t="n">
-        <v>428.1900024414062</v>
+        <v>432.3900146484375</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>8563.800048828125</v>
+        <v>8647.80029296875</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>0.03564138202803051</v>
+        <v>0.03553444227620745</v>
       </c>
       <c r="H3" s="9" t="n">
         <v>6893.1</v>
@@ -12224,13 +12777,13 @@
         <v>6893.1</v>
       </c>
       <c r="L3" s="9" t="n">
-        <v>1734.120048828125</v>
+        <v>1818.12029296875</v>
       </c>
       <c r="M3" s="15" t="n">
-        <v>0.2423728146738223</v>
+        <v>0.2545589492345605</v>
       </c>
       <c r="N3" s="15" t="n">
-        <v>0.2515733195265011</v>
+        <v>0.2637594540872393</v>
       </c>
       <c r="O3" s="7" t="n"/>
     </row>
@@ -12252,13 +12805,13 @@
         <v>150</v>
       </c>
       <c r="E4" s="10" t="n">
-        <v>74.33000183105469</v>
+        <v>72.05000305175781</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>11149.5002746582</v>
+        <v>10807.50045776367</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>0.04640271800426989</v>
+        <v>0.04440880780731467</v>
       </c>
       <c r="H4" s="9" t="n">
         <v>12219</v>
@@ -12273,13 +12826,13 @@
         <v>12219</v>
       </c>
       <c r="L4" s="9" t="n">
-        <v>-1069.499725341795</v>
+        <v>-1411.499542236326</v>
       </c>
       <c r="M4" s="15" t="n">
-        <v>-0.0875275984402812</v>
+        <v>-0.1155167806069504</v>
       </c>
       <c r="N4" s="15" t="n">
-        <v>-0.08752759844028114</v>
+        <v>-0.1155167806069504</v>
       </c>
       <c r="O4" s="7" t="n"/>
     </row>
@@ -12301,13 +12854,13 @@
         <v>20</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>377.489990234375</v>
+        <v>368.8299865722656</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>7549.7998046875</v>
+        <v>7376.599731445312</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>0.03142124962514032</v>
+        <v>0.03031098643256771</v>
       </c>
       <c r="H5" s="9" t="n">
         <v>22085.17</v>
@@ -12322,13 +12875,13 @@
         <v>9410.169999999998</v>
       </c>
       <c r="L5" s="9" t="n">
-        <v>-1860.370195312498</v>
+        <v>-2033.570268554686</v>
       </c>
       <c r="M5" s="15" t="n">
-        <v>-0.1976978306781385</v>
+        <v>-0.2161034570634416</v>
       </c>
       <c r="N5" s="15" t="n">
-        <v>-0.08423617274906638</v>
+        <v>-0.09207854268519038</v>
       </c>
       <c r="O5" s="7" t="n"/>
     </row>
@@ -12350,13 +12903,13 @@
         <v>600</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>14.98999977111816</v>
+        <v>16</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>8993.999862670898</v>
+        <v>9600</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>0.03743181569370865</v>
+        <v>0.03944710033705958</v>
       </c>
       <c r="H6" s="9" t="n">
         <v>11165</v>
@@ -12365,19 +12918,19 @@
         <v>6936</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>229.77</v>
+        <v>291</v>
       </c>
       <c r="K6" s="9" t="n">
         <v>4229</v>
       </c>
       <c r="L6" s="9" t="n">
-        <v>4994.769862670899</v>
+        <v>5662</v>
       </c>
       <c r="M6" s="15" t="n">
-        <v>1.126743878616907</v>
+        <v>1.270040198628518</v>
       </c>
       <c r="N6" s="15" t="n">
-        <v>0.4473595936113658</v>
+        <v>0.5071204657411554</v>
       </c>
       <c r="O6" s="7" t="n"/>
     </row>
@@ -12399,13 +12952,13 @@
         <v>107</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>221.5399932861328</v>
+        <v>235.25</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>23704.77928161621</v>
+        <v>25171.75</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>0.09865609769600341</v>
+        <v>0.1034325570738937</v>
       </c>
       <c r="H7" s="9" t="n">
         <v>28073.97</v>
@@ -12420,13 +12973,13 @@
         <v>28073.97</v>
       </c>
       <c r="L7" s="9" t="n">
-        <v>-4369.19071838379</v>
+        <v>-2902.220000000001</v>
       </c>
       <c r="M7" s="15" t="n">
-        <v>-0.1556313808978136</v>
+        <v>-0.1033776127850818</v>
       </c>
       <c r="N7" s="15" t="n">
-        <v>-0.1556313808978135</v>
+        <v>-0.1033776127850817</v>
       </c>
       <c r="O7" s="7" t="n"/>
     </row>
@@ -12448,13 +13001,13 @@
         <v>43</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>388.8399963378906</v>
+        <v>392.5400085449219</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>16720.1198425293</v>
+        <v>16879.22036743164</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>0.06958688613281989</v>
+        <v>0.06935794785889746</v>
       </c>
       <c r="H8" s="9" t="n">
         <v>17698.7</v>
@@ -12469,13 +13022,13 @@
         <v>17698.7</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>-915.9701574707033</v>
+        <v>-756.8696325683595</v>
       </c>
       <c r="M8" s="15" t="n">
-        <v>-0.05529107547281454</v>
+        <v>-0.04630168501462587</v>
       </c>
       <c r="N8" s="15" t="n">
-        <v>-0.05175352751731501</v>
+        <v>-0.04276413705912635</v>
       </c>
       <c r="O8" s="7" t="n"/>
     </row>
@@ -12497,13 +13050,13 @@
         <v>500</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>27.05999946594238</v>
+        <v>28.52000045776367</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>13529.99973297119</v>
+        <v>14260.00022888184</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>0.0563100360321894</v>
+        <v>0.05859538123283274</v>
       </c>
       <c r="H9" s="9" t="n">
         <v>12425</v>
@@ -12518,13 +13071,13 @@
         <v>12425</v>
       </c>
       <c r="L9" s="9" t="n">
-        <v>1104.999732971191</v>
+        <v>1835.000228881836</v>
       </c>
       <c r="M9" s="15" t="n">
-        <v>0.08893358011840569</v>
+        <v>0.1476861351212745</v>
       </c>
       <c r="N9" s="15" t="n">
-        <v>0.08893358011840574</v>
+        <v>0.1476861351212745</v>
       </c>
       <c r="O9" s="7" t="n"/>
     </row>
@@ -12546,13 +13099,13 @@
         <v>25</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>234.3999938964844</v>
+        <v>207.6900024414062</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>5859.999847412109</v>
+        <v>5192.250061035156</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>0.02438852986465931</v>
+        <v>0.02133533428466224</v>
       </c>
       <c r="H10" s="9" t="n">
         <v>5210</v>
@@ -12561,19 +13114,19 @@
         <v>0</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="K10" s="9" t="n">
         <v>5210</v>
       </c>
       <c r="L10" s="9" t="n">
-        <v>651.7498474121094</v>
+        <v>-14.24993896484375</v>
       </c>
       <c r="M10" s="15" t="n">
-        <v>0.1247600474879288</v>
+        <v>-0.00340689807386639</v>
       </c>
       <c r="N10" s="15" t="n">
-        <v>0.1250959400023243</v>
+        <v>-0.002735113045075576</v>
       </c>
       <c r="O10" s="7" t="n"/>
     </row>
@@ -12595,13 +13148,13 @@
         <v>430</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>37.09999847412109</v>
+        <v>38.34500122070312</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>15952.99934387207</v>
+        <v>16488.35052490234</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>0.06639423396926115</v>
+        <v>0.06775183516129497</v>
       </c>
       <c r="H11" s="9" t="n">
         <v>17180.9</v>
@@ -12616,13 +13169,13 @@
         <v>17180.9</v>
       </c>
       <c r="L11" s="9" t="n">
-        <v>-1087.390656127931</v>
+        <v>-552.0394750976593</v>
       </c>
       <c r="M11" s="15" t="n">
-        <v>-0.0714689367918987</v>
+        <v>-0.04030926640034335</v>
       </c>
       <c r="N11" s="15" t="n">
-        <v>-0.06329066906436397</v>
+        <v>-0.03213099867280871</v>
       </c>
       <c r="O11" s="7" t="n"/>
     </row>
@@ -12644,13 +13197,13 @@
         <v>200</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>23.40999984741211</v>
+        <v>23.89999961853027</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>4681.999969482422</v>
+        <v>4779.999923706055</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>0.01948585308111966</v>
+        <v>0.01964136839599686</v>
       </c>
       <c r="H12" s="9" t="n">
         <v>5947</v>
@@ -12665,13 +13218,13 @@
         <v>5947</v>
       </c>
       <c r="L12" s="9" t="n">
-        <v>-1218.800030517578</v>
+        <v>-1120.800076293945</v>
       </c>
       <c r="M12" s="15" t="n">
-        <v>-0.2127122970434804</v>
+        <v>-0.1962334078180503</v>
       </c>
       <c r="N12" s="15" t="n">
-        <v>-0.2049436742084376</v>
+        <v>-0.1884647849830075</v>
       </c>
       <c r="O12" s="7" t="n"/>
     </row>
@@ -12693,13 +13246,13 @@
         <v>120</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>128.2200012207031</v>
+        <v>125.9100036621094</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>15386.40014648438</v>
+        <v>15109.20043945312</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>0.06403612444595044</v>
+        <v>0.0620848068487346</v>
       </c>
       <c r="H13" s="9" t="n">
         <v>14520</v>
@@ -12714,13 +13267,13 @@
         <v>14520</v>
       </c>
       <c r="L13" s="9" t="n">
-        <v>1070.880146484375</v>
+        <v>793.6804394531246</v>
       </c>
       <c r="M13" s="15" t="n">
-        <v>0.05966943157605888</v>
+        <v>0.04057854266206095</v>
       </c>
       <c r="N13" s="15" t="n">
-        <v>0.07375207620415802</v>
+        <v>0.0546611872901601</v>
       </c>
       <c r="O13" s="7" t="n"/>
     </row>
@@ -12739,19 +13292,19 @@
         </is>
       </c>
       <c r="D14" s="13" t="n">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>141.6000061035156</v>
+        <v>127.2799987792969</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>5522.400238037109</v>
+        <v>7636.799926757812</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>0.02298348577422718</v>
+        <v>0.0313801680171734</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>17927.57</v>
+        <v>20737.43</v>
       </c>
       <c r="I14" s="9" t="n">
         <v>15703.6</v>
@@ -12760,16 +13313,16 @@
         <v>28</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>2223.969999999999</v>
+        <v>5033.83</v>
       </c>
       <c r="L14" s="9" t="n">
-        <v>3326.430238037108</v>
+        <v>2630.969926757811</v>
       </c>
       <c r="M14" s="15" t="n">
-        <v>1.483127127630818</v>
+        <v>0.5170953184270849</v>
       </c>
       <c r="N14" s="15" t="n">
-        <v>0.1855483056564335</v>
+        <v>0.1268705874719196</v>
       </c>
       <c r="O14" s="7" t="n"/>
     </row>
@@ -12791,13 +13344,13 @@
         <v>40</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>352.2000122070312</v>
+        <v>358.7200012207031</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>14088.00048828125</v>
+        <v>14348.80004882812</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>0.0586323599980154</v>
+        <v>0.05896026617109671</v>
       </c>
       <c r="H15" s="9" t="n">
         <v>12988</v>
@@ -12812,13 +13365,13 @@
         <v>12988</v>
       </c>
       <c r="L15" s="9" t="n">
-        <v>1118.76048828125</v>
+        <v>1379.560048828125</v>
       </c>
       <c r="M15" s="15" t="n">
-        <v>0.0846936008839891</v>
+        <v>0.1047736409630525</v>
       </c>
       <c r="N15" s="15" t="n">
-        <v>0.086138011108812</v>
+        <v>0.1062180511878754</v>
       </c>
       <c r="O15" s="7" t="n"/>
     </row>
@@ -12840,13 +13393,13 @@
         <v>200</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>84.55000305175781</v>
+        <v>84.55500030517578</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>16910.00061035156</v>
+        <v>16911.00006103516</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>0.07037714430642766</v>
+        <v>0.06948853293829942</v>
       </c>
       <c r="H16" s="9" t="n">
         <v>17734</v>
@@ -12855,19 +13408,19 @@
         <v>0</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>136.57</v>
+        <v>181.1</v>
       </c>
       <c r="K16" s="9" t="n">
         <v>17734</v>
       </c>
       <c r="L16" s="9" t="n">
-        <v>-687.4293896484378</v>
+        <v>-641.8999389648452</v>
       </c>
       <c r="M16" s="15" t="n">
-        <v>-0.04646438421385124</v>
+        <v>-0.04640802633161408</v>
       </c>
       <c r="N16" s="15" t="n">
-        <v>-0.03876335793664361</v>
+        <v>-0.03619600422718198</v>
       </c>
       <c r="O16" s="7" t="n"/>
     </row>
@@ -12889,13 +13442,13 @@
         <v>150</v>
       </c>
       <c r="E17" s="10" t="n">
-        <v>100.4599990844727</v>
+        <v>100.5749969482422</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>15068.9998626709</v>
+        <v>15086.24954223633</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>0.06271514722711061</v>
+        <v>0.06199049993776204</v>
       </c>
       <c r="H17" s="9" t="n">
         <v>16683</v>
@@ -12904,19 +13457,19 @@
         <v>1607.52</v>
       </c>
       <c r="J17" s="9" t="n">
-        <v>93.29000000000001</v>
+        <v>124.34</v>
       </c>
       <c r="K17" s="9" t="n">
         <v>15075.48</v>
       </c>
       <c r="L17" s="9" t="n">
-        <v>86.80986267089975</v>
+        <v>135.1095422363287</v>
       </c>
       <c r="M17" s="15" t="n">
-        <v>-0.0004298461693491978</v>
+        <v>0.0007143747486865589</v>
       </c>
       <c r="N17" s="15" t="n">
-        <v>0.005203492337762977</v>
+        <v>0.008098635871026117</v>
       </c>
       <c r="O17" s="7" t="n"/>
     </row>
@@ -12938,13 +13491,13 @@
         <v>150</v>
       </c>
       <c r="E18" s="10" t="n">
-        <v>49.63999938964844</v>
+        <v>50.5099983215332</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>7445.999908447266</v>
+        <v>7576.49974822998</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>0.03098924844163833</v>
+        <v>0.03113239018459736</v>
       </c>
       <c r="H18" s="9" t="n">
         <v>5769</v>
@@ -12959,13 +13512,13 @@
         <v>5769</v>
       </c>
       <c r="L18" s="9" t="n">
-        <v>1808.059908447266</v>
+        <v>1938.559748229981</v>
       </c>
       <c r="M18" s="15" t="n">
-        <v>0.2906916117953312</v>
+        <v>0.3133124888594176</v>
       </c>
       <c r="N18" s="15" t="n">
-        <v>0.3134095871810134</v>
+        <v>0.3360304642450998</v>
       </c>
       <c r="O18" s="7" t="n"/>
     </row>
@@ -12984,37 +13537,37 @@
         </is>
       </c>
       <c r="D19" s="13" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="E19" s="10" t="n">
-        <v>45.65000152587891</v>
+        <v>56.68999862670898</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>18260.00061035156</v>
+        <v>17006.9995880127</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>0.07599566242496143</v>
+        <v>0.06988300199798622</v>
       </c>
       <c r="H19" s="9" t="n">
         <v>18236.4</v>
       </c>
       <c r="I19" s="9" t="n">
-        <v>0</v>
+        <v>5630</v>
       </c>
       <c r="J19" s="9" t="n">
         <v>39.2</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>18236.4</v>
+        <v>12606.4</v>
       </c>
       <c r="L19" s="9" t="n">
-        <v>62.80061035156177</v>
+        <v>4439.799588012695</v>
       </c>
       <c r="M19" s="15" t="n">
-        <v>0.001294148535432545</v>
+        <v>0.3490766267937471</v>
       </c>
       <c r="N19" s="15" t="n">
-        <v>0.003443695595159229</v>
+        <v>0.2434581160762373</v>
       </c>
       <c r="O19" s="7" t="n"/>
     </row>
@@ -13036,13 +13589,13 @@
         <v>40</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>196.9299926757812</v>
+        <v>204.4149932861328</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>7877.19970703125</v>
+        <v>8176.599731445312</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>0.03278384390908443</v>
+        <v>0.03359824479398934</v>
       </c>
       <c r="H20" s="9" t="n">
         <v>8635</v>
@@ -13057,13 +13610,13 @@
         <v>8635</v>
       </c>
       <c r="L20" s="9" t="n">
-        <v>-757.80029296875</v>
+        <v>-458.4002685546875</v>
       </c>
       <c r="M20" s="15" t="n">
-        <v>-0.08775915378908512</v>
+        <v>-0.05308630788126086</v>
       </c>
       <c r="N20" s="15" t="n">
-        <v>-0.08775915378908512</v>
+        <v>-0.05308630788126086</v>
       </c>
       <c r="O20" s="7" t="n"/>
     </row>
@@ -13085,13 +13638,13 @@
         <v>10</v>
       </c>
       <c r="E21" s="10" t="n">
-        <v>535.3800048828125</v>
+        <v>518.1199951171875</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>5353.800048828125</v>
+        <v>5181.199951171875</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>0.02228179450173911</v>
+        <v>0.02128992857710887</v>
       </c>
       <c r="H21" s="9" t="n">
         <v>5069.8</v>
@@ -13106,13 +13659,13 @@
         <v>5069.8</v>
       </c>
       <c r="L21" s="9" t="n">
-        <v>284.0000488281248</v>
+        <v>111.3999511718748</v>
       </c>
       <c r="M21" s="15" t="n">
-        <v>0.05601799850647458</v>
+        <v>0.02197324375160259</v>
       </c>
       <c r="N21" s="15" t="n">
-        <v>0.05601799850647458</v>
+        <v>0.02197324375160259</v>
       </c>
       <c r="O21" s="7" t="n"/>
     </row>
@@ -13134,16 +13687,16 @@
         <v>38</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>443.4599914550781</v>
+        <v>450.7124938964844</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>16851.47967529297</v>
+        <v>17127.07476806641</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>0.07013358805906453</v>
+        <v>0.07037639967252468</v>
       </c>
       <c r="H22" s="9" t="n">
-        <v>14284.37917736824</v>
+        <v>14284.70668805384</v>
       </c>
       <c r="I22" s="9" t="n">
         <v>0</v>
@@ -13152,67 +13705,18 @@
         <v>51.6</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>14284.37917736824</v>
+        <v>14284.70668805384</v>
       </c>
       <c r="L22" s="9" t="n">
-        <v>2618.700497924729</v>
+        <v>2893.968080012561</v>
       </c>
       <c r="M22" s="15" t="n">
-        <v>0.1797138304751787</v>
+        <v>0.198979800011547</v>
       </c>
       <c r="N22" s="15" t="n">
-        <v>0.1833261680755242</v>
+        <v>0.2025920547905094</v>
       </c>
       <c r="O22" s="7" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>MBGL</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>Mobility Global Inc.</t>
-        </is>
-      </c>
-      <c r="D23" s="13" t="n">
-        <v>38</v>
-      </c>
-      <c r="E23" s="10" t="n">
-        <v>21.20000076293945</v>
-      </c>
-      <c r="F23" s="9" t="n">
-        <v>805.6000289916992</v>
-      </c>
-      <c r="G23" s="14" t="n">
-        <v>0.003352798784578661</v>
-      </c>
-      <c r="H23" s="9" t="n">
-        <v>729.7608226317609</v>
-      </c>
-      <c r="I23" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" s="9" t="n">
-        <v>729.7608226317609</v>
-      </c>
-      <c r="L23" s="9" t="n">
-        <v>75.83920635993832</v>
-      </c>
-      <c r="M23" s="15" t="n">
-        <v>0.1039233732587026</v>
-      </c>
-      <c r="N23" s="15" t="n">
-        <v>0.1039233732587025</v>
-      </c>
-      <c r="O23" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>